<commit_message>
UI/UX polish, bug fixes, and business logic refinement
</commit_message>
<xml_diff>
--- a/bookings.xlsx
+++ b/bookings.xlsx
@@ -397,17 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Job ID</v>
+        <v>Job_ID</v>
       </c>
       <c r="B1" t="str">
         <v>Date</v>
       </c>
       <c r="C1" t="str">
-        <v>Name</v>
+        <v>Customer</v>
       </c>
       <c r="D1" t="str">
         <v>Phone</v>
@@ -422,10 +422,10 @@
         <v>Issue</v>
       </c>
       <c r="H1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="I1" t="str">
         <v>Status</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Price</v>
       </c>
       <c r="J1" t="str">
         <v>Rating</v>
@@ -434,45 +434,20 @@
         <v>Review</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
-      <c r="A2" t="str">
-        <v>JOB-MSUAALWZ-QMKH</v>
-      </c>
+    <row r="2">
       <c r="B2" t="str">
-        <v>15/8/2026</v>
-      </c>
-      <c r="C2" t="str">
-        <v>satwick shaw</v>
-      </c>
-      <c r="D2" t="str">
-        <v>8250297411</v>
-      </c>
-      <c r="E2" t="str">
-        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
-      </c>
-      <c r="F2" t="str">
-        <v>AC</v>
-      </c>
-      <c r="G2" t="str" xml:space="preserve">
-        <v xml:space="preserve">isisi
-</v>
-      </c>
-      <c r="H2" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="I2">
-        <v>499</v>
+        <v>Invalid Date</v>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>JOB-MSUAC7QG-BXG5</v>
+        <v>JOB-MSUERQDN-IX1H</v>
       </c>
       <c r="B3" t="str">
         <v>15/8/2026</v>
@@ -490,94 +465,24 @@
         <v>AC</v>
       </c>
       <c r="G3" t="str">
-        <v>ew</v>
-      </c>
-      <c r="H3" t="str">
+        <v>d</v>
+      </c>
+      <c r="H3">
+        <v>499</v>
+      </c>
+      <c r="I3" t="str">
         <v>Completed</v>
       </c>
-      <c r="I3">
-        <v>499</v>
-      </c>
       <c r="J3" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
       <c r="K3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>JOB-MSUB1P5C-GKVF</v>
-      </c>
-      <c r="B4" t="str">
-        <v>15/8/2026</v>
-      </c>
-      <c r="C4" t="str">
-        <v>satyyy</v>
-      </c>
-      <c r="D4" t="str">
-        <v>8250297411</v>
-      </c>
-      <c r="E4" t="str">
-        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
-      </c>
-      <c r="F4" t="str">
-        <v>AC</v>
-      </c>
-      <c r="G4" t="str">
-        <v>dfdfdd</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="I4">
-        <v>499</v>
-      </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>JOB-MSUC2RLU-S7QW</v>
-      </c>
-      <c r="B5" t="str">
-        <v>15/8/2026</v>
-      </c>
-      <c r="C5" t="str">
-        <v>zxzX</v>
-      </c>
-      <c r="D5" t="str">
-        <v>8250297411</v>
-      </c>
-      <c r="E5" t="str">
-        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
-      </c>
-      <c r="F5" t="str">
-        <v>Fridge</v>
-      </c>
-      <c r="G5" t="str">
-        <v>xzzzzzzzz</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Pending</v>
-      </c>
-      <c r="I5">
-        <v>299</v>
-      </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
-        <v/>
+        <v>N/A</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement enterprise worker portal features
</commit_message>
<xml_diff>
--- a/bookings.xlsx
+++ b/bookings.xlsx
@@ -1,41 +1,115 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satwi\OneDrive\Desktop\project\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CAB4A3-66F6-40CC-99E5-CB6C06485180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Bookings" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+  <si>
+    <t>Job_ID</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Customer</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Appliance</t>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>Invalid Date</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>JOB-MSUERQDN-IX1H</t>
+  </si>
+  <si>
+    <t>15/8/2026</t>
+  </si>
+  <si>
+    <t>sat</t>
+  </si>
+  <si>
+    <t>8250297411</t>
+  </si>
+  <si>
+    <t xml:space="preserve">160/21 guru teg bahadur nagar </t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>AC-83799A</t>
+  </si>
+  <si>
+    <t>Satwick</t>
+  </si>
+  <si>
+    <t>9832731345</t>
+  </si>
+  <si>
+    <t>guru teg bahadur nagar</t>
+  </si>
+  <si>
+    <t>Tggg</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -72,6 +146,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,93 +478,137 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.796875" customWidth="1"/>
+    <col min="2" max="2" width="17.09765625" customWidth="1"/>
+    <col min="3" max="3" width="14.3984375" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="26.3984375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Job_ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Date</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Customer</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Phone</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Address</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Appliance</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Issue</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Price</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Rating</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Review</v>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="2">
-      <c r="B2" t="str">
-        <v>Invalid Date</v>
-      </c>
-      <c r="J2" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K2" t="str">
-        <v>N/A</v>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>JOB-MSUERQDN-IX1H</v>
-      </c>
-      <c r="B3" t="str">
-        <v>15/8/2026</v>
-      </c>
-      <c r="C3" t="str">
-        <v>sat</v>
-      </c>
-      <c r="D3" t="str">
-        <v>8250297411</v>
-      </c>
-      <c r="E3" t="str">
-        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
-      </c>
-      <c r="F3" t="str">
-        <v>AC</v>
-      </c>
-      <c r="G3" t="str">
-        <v>d</v>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
       </c>
       <c r="H3">
         <v>499</v>
       </c>
-      <c r="I3" t="str">
-        <v>Completed</v>
-      </c>
-      <c r="J3" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="K3" t="str">
-        <v>N/A</v>
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4">
+        <v>499</v>
+      </c>
+      <c r="I4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError sqref="A1:K2 B4:K4 B3:K3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: live tracking with On the Way & Reached Location stages and real-time checklist sync
</commit_message>
<xml_diff>
--- a/bookings.xlsx
+++ b/bookings.xlsx
@@ -1,115 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satwi\OneDrive\Desktop\project\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CAB4A3-66F6-40CC-99E5-CB6C06485180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
   <sheets>
     <sheet name="Bookings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
-  <si>
-    <t>Job_ID</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>Appliance</t>
-  </si>
-  <si>
-    <t>Issue</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Rating</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>Invalid Date</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>JOB-MSUERQDN-IX1H</t>
-  </si>
-  <si>
-    <t>15/8/2026</t>
-  </si>
-  <si>
-    <t>sat</t>
-  </si>
-  <si>
-    <t>8250297411</t>
-  </si>
-  <si>
-    <t xml:space="preserve">160/21 guru teg bahadur nagar </t>
-  </si>
-  <si>
-    <t>AC</t>
-  </si>
-  <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>AC-83799A</t>
-  </si>
-  <si>
-    <t>Satwick</t>
-  </si>
-  <si>
-    <t>9832731345</t>
-  </si>
-  <si>
-    <t>guru teg bahadur nagar</t>
-  </si>
-  <si>
-    <t>Tggg</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -146,14 +72,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -478,137 +396,338 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="22.796875" customWidth="1"/>
-    <col min="2" max="2" width="17.09765625" customWidth="1"/>
-    <col min="3" max="3" width="14.3984375" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="26.3984375" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K10"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="J2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Job_ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Customer</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Address</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Appliance</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Issue</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Price</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Rating</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Review</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="str">
+        <v>Invalid Date</v>
+      </c>
+      <c r="J2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K2" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>JOB-MSUERQDN-IX1H</v>
+      </c>
+      <c r="B3" t="str">
+        <v>15/8/2026</v>
+      </c>
+      <c r="C3" t="str">
+        <v>sat</v>
+      </c>
+      <c r="D3" t="str">
+        <v>8250297411</v>
+      </c>
+      <c r="E3" t="str">
+        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
+      </c>
+      <c r="F3" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G3" t="str">
+        <v>d</v>
       </c>
       <c r="H3">
         <v>499</v>
       </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>25</v>
+      <c r="I3" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J3" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K3" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>AC-83799A</v>
+      </c>
+      <c r="B4" t="str">
+        <v>15/8/2026</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Satwick</v>
+      </c>
+      <c r="D4" t="str">
+        <v>9832731345</v>
+      </c>
+      <c r="E4" t="str">
+        <v>guru teg bahadur nagar</v>
+      </c>
+      <c r="F4" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Tggg</v>
       </c>
       <c r="H4">
         <v>499</v>
       </c>
-      <c r="I4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" t="s">
-        <v>12</v>
-      </c>
-      <c r="K4" t="s">
-        <v>12</v>
+      <c r="I4" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J4" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K4" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>AC-93169J</v>
+      </c>
+      <c r="B5" t="str">
+        <v>15/8/2026</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Supreme</v>
+      </c>
+      <c r="D5" t="str">
+        <v>7908443121</v>
+      </c>
+      <c r="E5" t="str">
+        <v>asasadaa</v>
+      </c>
+      <c r="F5" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G5" t="str">
+        <v>sdadadadadad</v>
+      </c>
+      <c r="H5">
+        <v>499</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Technician Assigned</v>
+      </c>
+      <c r="J5" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K5" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>AC-11887N</v>
+      </c>
+      <c r="B6" t="str">
+        <v>15/8/2026</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="D6" t="str">
+        <v>7908443121</v>
+      </c>
+      <c r="E6" t="str">
+        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
+      </c>
+      <c r="F6" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G6" t="str">
+        <v>aasdd</v>
+      </c>
+      <c r="H6">
+        <v>499</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Work in Progress</v>
+      </c>
+      <c r="J6" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K6" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>FR-74461S</v>
+      </c>
+      <c r="B7" t="str">
+        <v>15/8/2026</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Satwick</v>
+      </c>
+      <c r="D7" t="str">
+        <v>9832731345</v>
+      </c>
+      <c r="E7" t="str">
+        <v>guru teg bahadur nagar</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Fridge</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Ttgg</v>
+      </c>
+      <c r="H7">
+        <v>299</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J7" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K7" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AC-81394E</v>
+      </c>
+      <c r="B8" t="str">
+        <v>16/8/2026</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Supreme</v>
+      </c>
+      <c r="D8" t="str">
+        <v>7908443121</v>
+      </c>
+      <c r="E8" t="str">
+        <v xml:space="preserve">160/21 guru teg bahadur nagar </v>
+      </c>
+      <c r="F8" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G8" t="str">
+        <v xml:space="preserve">not working properly and is making noise </v>
+      </c>
+      <c r="H8">
+        <v>499</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J8" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K8" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AC-93930I</v>
+      </c>
+      <c r="B9" t="str">
+        <v>16/8/2026</v>
+      </c>
+      <c r="C9" t="str">
+        <v xml:space="preserve">Satwick Shaw </v>
+      </c>
+      <c r="D9" t="str">
+        <v>9832731345</v>
+      </c>
+      <c r="E9" t="str">
+        <v>guru teg bahadur nagar</v>
+      </c>
+      <c r="F9" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G9" t="str">
+        <v xml:space="preserve">I have faulty fans </v>
+      </c>
+      <c r="H9">
+        <v>499</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K9" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>AC-73488N</v>
+      </c>
+      <c r="B10" t="str">
+        <v>17/8/2026</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Ankit Majhi</v>
+      </c>
+      <c r="D10" t="str">
+        <v>6294125531</v>
+      </c>
+      <c r="E10" t="str">
+        <v>bencahity</v>
+      </c>
+      <c r="F10" t="str">
+        <v>AC</v>
+      </c>
+      <c r="G10" t="str">
+        <v>ami gay ho</v>
+      </c>
+      <c r="H10">
+        <v>499</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Completed</v>
+      </c>
+      <c r="J10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="K10" t="str">
+        <v>N/A</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:K2 B4:K4 B3:K3" numberStoredAsText="1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>